<commit_message>
Introduction lecture more or less done.
</commit_message>
<xml_diff>
--- a/slides/schedule.xlsx
+++ b/slides/schedule.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\gitlab\mop-lecture_notes\slides\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{2D907072-1FB7-4EB3-AE6F-31DCF52FEB0C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{52A9F945-78D1-4AF9-8AD8-386EC4F634F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="23520" xr2:uid="{FA211EDD-E1F2-42CA-9429-48F7FEBA2EEC}"/>
+    <workbookView xWindow="17100" yWindow="4920" windowWidth="29700" windowHeight="23550" xr2:uid="{FA211EDD-E1F2-42CA-9429-48F7FEBA2EEC}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -123,7 +123,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -134,6 +134,13 @@
     <font>
       <b/>
       <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
@@ -388,13 +395,7 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -406,19 +407,13 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -427,26 +422,14 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="12" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="13" xfId="0" applyFill="1" applyBorder="1"/>
@@ -468,17 +451,41 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="10" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -827,435 +834,439 @@
   <sheetData>
     <row r="11" spans="9:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="12" spans="9:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="I12" s="5" t="s">
+      <c r="I12" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="J12" s="6" t="s">
+      <c r="J12" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="K12" s="6" t="s">
+      <c r="K12" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="L12" s="6" t="s">
+      <c r="L12" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="M12" s="6" t="s">
+      <c r="M12" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="N12" s="6" t="s">
+      <c r="N12" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="O12" s="6" t="s">
+      <c r="O12" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="P12" s="7" t="s">
+      <c r="P12" s="5" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="13" spans="9:16" x14ac:dyDescent="0.25">
-      <c r="I13" s="8">
+      <c r="I13" s="23">
         <v>1</v>
       </c>
-      <c r="J13" s="24">
+      <c r="J13" s="16">
         <v>19</v>
       </c>
-      <c r="K13" s="25">
+      <c r="K13" s="17">
         <v>20</v>
       </c>
-      <c r="L13" s="25">
+      <c r="L13" s="17">
         <v>21</v>
       </c>
-      <c r="M13" s="25">
+      <c r="M13" s="17">
         <v>22</v>
       </c>
-      <c r="N13" s="25">
+      <c r="N13" s="17">
         <v>23</v>
       </c>
-      <c r="O13" s="25">
+      <c r="O13" s="17">
         <v>24</v>
       </c>
-      <c r="P13" s="26">
+      <c r="P13" s="18">
         <v>25</v>
       </c>
     </row>
     <row r="14" spans="9:16" ht="75.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="I14" s="8"/>
-      <c r="J14" s="27"/>
-      <c r="K14" s="11" t="s">
+      <c r="I14" s="23"/>
+      <c r="J14" s="19"/>
+      <c r="K14" s="31" t="s">
         <v>2</v>
       </c>
-      <c r="L14" s="10"/>
-      <c r="M14" s="10"/>
-      <c r="N14" s="11" t="s">
+      <c r="L14" s="7"/>
+      <c r="M14" s="7"/>
+      <c r="N14" s="31" t="s">
         <v>3</v>
       </c>
-      <c r="O14" s="12"/>
-      <c r="P14" s="13"/>
+      <c r="O14" s="8"/>
+      <c r="P14" s="9"/>
     </row>
     <row r="15" spans="9:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="I15" s="8">
+      <c r="I15" s="23">
         <v>2</v>
       </c>
-      <c r="J15" s="28">
+      <c r="J15" s="20">
         <v>26</v>
       </c>
-      <c r="K15" s="9">
+      <c r="K15" s="6">
         <v>27</v>
       </c>
-      <c r="L15" s="9">
+      <c r="L15" s="6">
         <v>28</v>
       </c>
-      <c r="M15" s="9">
+      <c r="M15" s="6">
         <v>29</v>
       </c>
-      <c r="N15" s="9">
+      <c r="N15" s="6">
         <v>30</v>
       </c>
-      <c r="O15" s="9">
+      <c r="O15" s="6">
         <v>31</v>
       </c>
-      <c r="P15" s="14">
+      <c r="P15" s="10">
         <v>1</v>
       </c>
     </row>
     <row r="16" spans="9:16" ht="72.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="I16" s="8"/>
-      <c r="J16" s="27"/>
-      <c r="K16" s="11" t="s">
+      <c r="I16" s="23"/>
+      <c r="J16" s="19"/>
+      <c r="K16" s="31" t="s">
         <v>4</v>
       </c>
-      <c r="L16" s="10"/>
-      <c r="M16" s="10"/>
-      <c r="N16" s="11" t="s">
+      <c r="L16" s="7"/>
+      <c r="M16" s="7"/>
+      <c r="N16" s="31" t="s">
         <v>5</v>
       </c>
-      <c r="O16" s="12"/>
+      <c r="O16" s="8"/>
       <c r="P16" s="1" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="17" spans="9:16" x14ac:dyDescent="0.25">
-      <c r="I17" s="8">
+      <c r="I17" s="23">
         <v>3</v>
       </c>
-      <c r="J17" s="29">
+      <c r="J17" s="21">
         <v>2</v>
       </c>
-      <c r="K17" s="15">
+      <c r="K17" s="11">
         <v>3</v>
       </c>
-      <c r="L17" s="15">
+      <c r="L17" s="11">
         <v>4</v>
       </c>
-      <c r="M17" s="15">
+      <c r="M17" s="11">
         <v>5</v>
       </c>
-      <c r="N17" s="15">
+      <c r="N17" s="11">
         <v>6</v>
       </c>
-      <c r="O17" s="15">
+      <c r="O17" s="11">
         <v>7</v>
       </c>
-      <c r="P17" s="14">
+      <c r="P17" s="10">
         <v>8</v>
       </c>
     </row>
     <row r="18" spans="9:16" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="I18" s="8"/>
-      <c r="J18" s="27"/>
-      <c r="K18" s="11" t="s">
+      <c r="I18" s="23"/>
+      <c r="J18" s="19"/>
+      <c r="K18" s="31" t="s">
         <v>6</v>
       </c>
-      <c r="L18" s="10"/>
-      <c r="M18" s="10"/>
-      <c r="N18" s="11" t="s">
+      <c r="L18" s="7"/>
+      <c r="M18" s="7"/>
+      <c r="N18" s="31" t="s">
         <v>7</v>
       </c>
-      <c r="O18" s="12"/>
-      <c r="P18" s="13"/>
+      <c r="O18" s="8"/>
+      <c r="P18" s="9"/>
     </row>
     <row r="19" spans="9:16" ht="36.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="I19" s="8"/>
-      <c r="J19" s="30" t="s">
+      <c r="I19" s="23"/>
+      <c r="J19" s="25" t="s">
         <v>15</v>
       </c>
-      <c r="K19" s="2"/>
-      <c r="L19" s="2"/>
-      <c r="M19" s="2"/>
-      <c r="N19" s="3"/>
-      <c r="O19" s="12"/>
-      <c r="P19" s="13"/>
+      <c r="K19" s="26"/>
+      <c r="L19" s="26"/>
+      <c r="M19" s="26"/>
+      <c r="N19" s="27"/>
+      <c r="O19" s="8"/>
+      <c r="P19" s="9"/>
     </row>
     <row r="20" spans="9:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="I20" s="8">
+      <c r="I20" s="23">
         <v>4</v>
       </c>
-      <c r="J20" s="29">
+      <c r="J20" s="21">
         <v>9</v>
       </c>
-      <c r="K20" s="15">
+      <c r="K20" s="11">
         <v>10</v>
       </c>
-      <c r="L20" s="15">
+      <c r="L20" s="11">
         <v>11</v>
       </c>
-      <c r="M20" s="15">
+      <c r="M20" s="11">
         <v>12</v>
       </c>
-      <c r="N20" s="15">
+      <c r="N20" s="11">
         <v>13</v>
       </c>
-      <c r="O20" s="15">
+      <c r="O20" s="11">
         <v>14</v>
       </c>
-      <c r="P20" s="14">
+      <c r="P20" s="10">
         <v>15</v>
       </c>
     </row>
     <row r="21" spans="9:16" ht="72.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="I21" s="8"/>
-      <c r="J21" s="31" t="s">
+      <c r="I21" s="23"/>
+      <c r="J21" s="32" t="s">
         <v>14</v>
       </c>
-      <c r="K21" s="11" t="s">
+      <c r="K21" s="31" t="s">
         <v>8</v>
       </c>
-      <c r="L21" s="10"/>
-      <c r="M21" s="10"/>
-      <c r="N21" s="10"/>
-      <c r="O21" s="12"/>
+      <c r="L21" s="7"/>
+      <c r="M21" s="7"/>
+      <c r="N21" s="7"/>
+      <c r="O21" s="8"/>
       <c r="P21" s="1" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="22" spans="9:16" x14ac:dyDescent="0.25">
-      <c r="I22" s="8">
+      <c r="I22" s="23">
         <v>5</v>
       </c>
-      <c r="J22" s="29">
+      <c r="J22" s="21">
         <v>16</v>
       </c>
-      <c r="K22" s="15">
+      <c r="K22" s="11">
         <v>17</v>
       </c>
-      <c r="L22" s="15">
+      <c r="L22" s="11">
         <v>18</v>
       </c>
-      <c r="M22" s="15">
+      <c r="M22" s="11">
         <v>19</v>
       </c>
-      <c r="N22" s="15">
+      <c r="N22" s="11">
         <v>20</v>
       </c>
-      <c r="O22" s="15">
+      <c r="O22" s="11">
         <v>21</v>
       </c>
-      <c r="P22" s="14">
+      <c r="P22" s="10">
         <v>22</v>
       </c>
     </row>
     <row r="23" spans="9:16" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="I23" s="8"/>
-      <c r="J23" s="27"/>
-      <c r="K23" s="11" t="s">
+      <c r="I23" s="23"/>
+      <c r="J23" s="19"/>
+      <c r="K23" s="31" t="s">
         <v>9</v>
       </c>
-      <c r="L23" s="10"/>
-      <c r="M23" s="10"/>
-      <c r="N23" s="11" t="s">
+      <c r="L23" s="7"/>
+      <c r="M23" s="7"/>
+      <c r="N23" s="31" t="s">
         <v>10</v>
       </c>
-      <c r="O23" s="12"/>
-      <c r="P23" s="13"/>
+      <c r="O23" s="8"/>
+      <c r="P23" s="9"/>
     </row>
     <row r="24" spans="9:16" ht="36.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="I24" s="8"/>
-      <c r="J24" s="30" t="s">
+      <c r="I24" s="23"/>
+      <c r="J24" s="25" t="s">
         <v>16</v>
       </c>
-      <c r="K24" s="2"/>
-      <c r="L24" s="2"/>
-      <c r="M24" s="2"/>
-      <c r="N24" s="3"/>
-      <c r="O24" s="12"/>
-      <c r="P24" s="13"/>
+      <c r="K24" s="26"/>
+      <c r="L24" s="26"/>
+      <c r="M24" s="26"/>
+      <c r="N24" s="27"/>
+      <c r="O24" s="8"/>
+      <c r="P24" s="9"/>
     </row>
     <row r="25" spans="9:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="I25" s="8">
+      <c r="I25" s="23">
         <v>6</v>
       </c>
-      <c r="J25" s="29">
+      <c r="J25" s="21">
         <v>23</v>
       </c>
-      <c r="K25" s="15">
+      <c r="K25" s="11">
         <v>24</v>
       </c>
-      <c r="L25" s="15">
+      <c r="L25" s="11">
         <v>25</v>
       </c>
-      <c r="M25" s="15">
+      <c r="M25" s="11">
         <v>26</v>
       </c>
-      <c r="N25" s="15">
+      <c r="N25" s="11">
         <v>27</v>
       </c>
-      <c r="O25" s="15">
+      <c r="O25" s="11">
         <v>28</v>
       </c>
-      <c r="P25" s="17">
+      <c r="P25" s="12">
         <v>1</v>
       </c>
     </row>
     <row r="26" spans="9:16" ht="72.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="I26" s="8"/>
-      <c r="J26" s="27"/>
-      <c r="K26" s="11" t="s">
+      <c r="I26" s="23"/>
+      <c r="J26" s="19"/>
+      <c r="K26" s="31" t="s">
         <v>11</v>
       </c>
-      <c r="L26" s="10"/>
-      <c r="M26" s="10"/>
-      <c r="N26" s="16" t="s">
+      <c r="L26" s="7"/>
+      <c r="M26" s="7"/>
+      <c r="N26" s="33" t="s">
         <v>14</v>
       </c>
-      <c r="O26" s="12"/>
+      <c r="O26" s="8"/>
       <c r="P26" s="1" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="27" spans="9:16" x14ac:dyDescent="0.25">
-      <c r="I27" s="8">
+      <c r="I27" s="23">
         <v>7</v>
       </c>
-      <c r="J27" s="32">
+      <c r="J27" s="22">
         <v>2</v>
       </c>
-      <c r="K27" s="18">
+      <c r="K27" s="13">
         <v>3</v>
       </c>
-      <c r="L27" s="18">
+      <c r="L27" s="13">
         <v>4</v>
       </c>
-      <c r="M27" s="18">
+      <c r="M27" s="13">
         <v>5</v>
       </c>
-      <c r="N27" s="18">
+      <c r="N27" s="13">
         <v>6</v>
       </c>
-      <c r="O27" s="18">
+      <c r="O27" s="13">
         <v>7</v>
       </c>
-      <c r="P27" s="17">
+      <c r="P27" s="12">
         <v>8</v>
       </c>
     </row>
     <row r="28" spans="9:16" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="I28" s="8"/>
-      <c r="J28" s="27"/>
-      <c r="K28" s="11" t="s">
+      <c r="I28" s="23"/>
+      <c r="J28" s="19"/>
+      <c r="K28" s="31" t="s">
         <v>12</v>
       </c>
-      <c r="L28" s="10"/>
-      <c r="M28" s="10"/>
-      <c r="N28" s="16" t="s">
+      <c r="L28" s="7"/>
+      <c r="M28" s="7"/>
+      <c r="N28" s="33" t="s">
         <v>14</v>
       </c>
-      <c r="O28" s="12"/>
-      <c r="P28" s="13"/>
+      <c r="O28" s="8"/>
+      <c r="P28" s="9"/>
     </row>
     <row r="29" spans="9:16" ht="36.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="I29" s="8"/>
-      <c r="J29" s="30" t="s">
+      <c r="I29" s="23"/>
+      <c r="J29" s="25" t="s">
         <v>17</v>
       </c>
-      <c r="K29" s="2"/>
-      <c r="L29" s="2"/>
-      <c r="M29" s="2"/>
-      <c r="N29" s="3"/>
-      <c r="O29" s="12"/>
-      <c r="P29" s="13"/>
+      <c r="K29" s="26"/>
+      <c r="L29" s="26"/>
+      <c r="M29" s="26"/>
+      <c r="N29" s="27"/>
+      <c r="O29" s="8"/>
+      <c r="P29" s="9"/>
     </row>
     <row r="30" spans="9:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="I30" s="8">
+      <c r="I30" s="23">
         <v>8</v>
       </c>
-      <c r="J30" s="32">
+      <c r="J30" s="22">
         <v>9</v>
       </c>
-      <c r="K30" s="18">
+      <c r="K30" s="13">
         <v>10</v>
       </c>
-      <c r="L30" s="18">
+      <c r="L30" s="13">
         <v>11</v>
       </c>
-      <c r="M30" s="18">
+      <c r="M30" s="13">
         <v>12</v>
       </c>
-      <c r="N30" s="18">
+      <c r="N30" s="13">
         <v>13</v>
       </c>
-      <c r="O30" s="18">
+      <c r="O30" s="13">
         <v>14</v>
       </c>
-      <c r="P30" s="17">
+      <c r="P30" s="12">
         <v>15</v>
       </c>
     </row>
     <row r="31" spans="9:16" ht="82.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="I31" s="8"/>
-      <c r="J31" s="27"/>
-      <c r="K31" s="11" t="s">
+      <c r="I31" s="23"/>
+      <c r="J31" s="19"/>
+      <c r="K31" s="31" t="s">
         <v>13</v>
       </c>
-      <c r="L31" s="10"/>
-      <c r="M31" s="10"/>
-      <c r="N31" s="16" t="s">
+      <c r="L31" s="7"/>
+      <c r="M31" s="7"/>
+      <c r="N31" s="33" t="s">
         <v>14</v>
       </c>
-      <c r="O31" s="4" t="s">
+      <c r="O31" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="P31" s="13"/>
+      <c r="P31" s="9"/>
     </row>
     <row r="32" spans="9:16" x14ac:dyDescent="0.25">
-      <c r="I32" s="8">
+      <c r="I32" s="23">
         <v>9</v>
       </c>
-      <c r="J32" s="32">
+      <c r="J32" s="22">
         <v>16</v>
       </c>
-      <c r="K32" s="18">
+      <c r="K32" s="13">
         <v>17</v>
       </c>
-      <c r="L32" s="18">
+      <c r="L32" s="13">
         <v>18</v>
       </c>
-      <c r="M32" s="18">
+      <c r="M32" s="13">
         <v>19</v>
       </c>
-      <c r="N32" s="18">
+      <c r="N32" s="13">
         <v>20</v>
       </c>
-      <c r="O32" s="18">
+      <c r="O32" s="13">
         <v>21</v>
       </c>
-      <c r="P32" s="17">
+      <c r="P32" s="12">
         <v>22</v>
       </c>
     </row>
     <row r="33" spans="9:16" ht="36.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="I33" s="19"/>
-      <c r="J33" s="33" t="s">
+      <c r="I33" s="24"/>
+      <c r="J33" s="28" t="s">
         <v>23</v>
       </c>
-      <c r="K33" s="20"/>
-      <c r="L33" s="20"/>
-      <c r="M33" s="20"/>
-      <c r="N33" s="21"/>
-      <c r="O33" s="22"/>
-      <c r="P33" s="23"/>
+      <c r="K33" s="29"/>
+      <c r="L33" s="29"/>
+      <c r="M33" s="29"/>
+      <c r="N33" s="30"/>
+      <c r="O33" s="14"/>
+      <c r="P33" s="15"/>
     </row>
   </sheetData>
   <mergeCells count="13">
+    <mergeCell ref="J19:N19"/>
+    <mergeCell ref="J24:N24"/>
+    <mergeCell ref="J29:N29"/>
+    <mergeCell ref="J33:N33"/>
     <mergeCell ref="I25:I26"/>
     <mergeCell ref="I27:I29"/>
     <mergeCell ref="I30:I31"/>
@@ -1265,10 +1276,6 @@
     <mergeCell ref="I17:I19"/>
     <mergeCell ref="I20:I21"/>
     <mergeCell ref="I22:I24"/>
-    <mergeCell ref="J19:N19"/>
-    <mergeCell ref="J24:N24"/>
-    <mergeCell ref="J29:N29"/>
-    <mergeCell ref="J33:N33"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="8" scale="74" orientation="landscape" r:id="rId1"/>

</xml_diff>